<commit_message>
fix(atlas): complete grouped header and certification coverage
</commit_message>
<xml_diff>
--- a/docs/testing/artifacts/atlas-document-school-grouping-02/native-qa/Dispatch-explicit-Vinh-Tan-NATIVE-SAVE-TEST-ONLY.xlsx
+++ b/docs/testing/artifacts/atlas-document-school-grouping-02/native-qa/Dispatch-explicit-Vinh-Tan-NATIVE-SAVE-TEST-ONLY.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D590B1E3-91DE-4A33-B25D-F1CEF6946144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C23EA13-D10D-461F-B7C9-85428B9B673B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -812,7 +812,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>3</v>
       </c>

</xml_diff>